<commit_message>
04182026 - Fix routers and ip address module.
</commit_message>
<xml_diff>
--- a/Inventory/assets/files/ip_export.xlsx
+++ b/Inventory/assets/files/ip_export.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IMPORTANT\Wifi-Inventory\Inventory\assets\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C544F8A6-EF44-49D5-9305-201466621ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE81B93D-ED37-49EE-879F-B306988BB1A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{1DA5F532-4404-45CC-8572-7A2C29C8382C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1DA5F532-4404-45CC-8572-7A2C29C8382C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Time:</t>
   </si>
@@ -89,14 +89,29 @@
     <t>Up State:</t>
   </si>
   <si>
-    <t>Down State</t>
+    <t>Subnet Mask:</t>
+  </si>
+  <si>
+    <t>255.255.255.0 /24</t>
+  </si>
+  <si>
+    <t>*Subnet Mask Format:</t>
+  </si>
+  <si>
+    <t>Down State:</t>
+  </si>
+  <si>
+    <t>Router Name:</t>
+  </si>
+  <si>
+    <t>Router IP:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,6 +123,21 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0" tint="-0.499984740745262"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -133,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -159,6 +189,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -166,6 +199,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -503,10 +539,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87101143-02CB-4335-BC89-C7FA34165B01}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="16.85546875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="22" style="3" customWidth="1"/>
     <col min="3" max="6" width="21" style="3" customWidth="1"/>
     <col min="7" max="7" width="16.85546875" style="3" customWidth="1"/>
     <col min="8" max="10" width="17.85546875" style="3" customWidth="1"/>
@@ -519,37 +556,37 @@
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
+      <c r="A4" s="1"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -559,39 +596,43 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-    </row>
-    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-    </row>
-    <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>16</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="13"/>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="5"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -599,63 +640,111 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="11" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+    </row>
+    <row r="10" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+    </row>
+    <row r="15" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B15" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G15" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H15" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I15" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="6" t="s">
+      <c r="J15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="K11" s="7" t="s">
+      <c r="K15" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="11">
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B13:G13"/>
     <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B10:G10"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B9:G9"/>
     <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="E7:F7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>